<commit_message>
fix download template and filter
</commit_message>
<xml_diff>
--- a/app/templates/Inventory_Product_Import_Template.xlsx
+++ b/app/templates/Inventory_Product_Import_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lapto\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WebSource\eng-promise\promise-inventory\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A6A28B-4828-4F02-A5A2-37D03D8FD67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18BCECDC-1F72-4D9D-95C5-7883C09F6C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62AADBC6-8410-49F7-A504-0FB573E6F6A1}"/>
   </bookViews>
@@ -1403,7 +1403,31 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -1414,18 +1438,6 @@
     <xf numFmtId="15" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1435,22 +1447,19 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1462,26 +1471,17 @@
     <xf numFmtId="15" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1574,8 +1574,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8620125" y="20926425"/>
-          <a:ext cx="0" cy="1504279"/>
+          <a:off x="8656320" y="20855940"/>
+          <a:ext cx="0" cy="1493801"/>
           <a:chOff x="63665100" y="150342600"/>
           <a:chExt cx="1016508" cy="908966"/>
         </a:xfrm>
@@ -1705,8 +1705,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8620125" y="11353800"/>
-          <a:ext cx="0" cy="1504279"/>
+          <a:off x="8656320" y="11346180"/>
+          <a:ext cx="0" cy="1493801"/>
           <a:chOff x="63665100" y="150342600"/>
           <a:chExt cx="1016508" cy="908966"/>
         </a:xfrm>
@@ -8056,50 +8056,50 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="51" t="s">
+      <c r="G1" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="51"/>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
-      <c r="K1" s="51"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="51"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
-      <c r="V1" s="51"/>
-      <c r="W1" s="51"/>
-      <c r="X1" s="51"/>
-      <c r="Y1" s="51"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
+      <c r="O1" s="36"/>
+      <c r="P1" s="36"/>
+      <c r="Q1" s="36"/>
+      <c r="R1" s="36"/>
+      <c r="S1" s="36"/>
+      <c r="T1" s="36"/>
+      <c r="U1" s="36"/>
+      <c r="V1" s="36"/>
+      <c r="W1" s="36"/>
+      <c r="X1" s="36"/>
+      <c r="Y1" s="36"/>
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:42" s="5" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="42" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="52" t="s">
+      <c r="B2" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="52" t="s">
+      <c r="D2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="52" t="s">
+      <c r="E2" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="52" t="s">
+      <c r="F2" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="52" t="s">
+      <c r="G2" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="48" t="s">
+      <c r="H2" s="32" t="s">
         <v>4</v>
       </c>
       <c r="I2" s="43" t="s">
@@ -8118,13 +8118,13 @@
       <c r="T2" s="44"/>
       <c r="U2" s="44"/>
       <c r="V2" s="44"/>
-      <c r="W2" s="45" t="s">
+      <c r="W2" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="X2" s="29" t="s">
+      <c r="X2" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="Y2" s="32" t="s">
+      <c r="Y2" s="45" t="s">
         <v>7</v>
       </c>
       <c r="Z2" s="43" t="s">
@@ -8143,207 +8143,207 @@
       <c r="AK2" s="44"/>
       <c r="AL2" s="44"/>
       <c r="AM2" s="44"/>
-      <c r="AN2" s="45" t="s">
+      <c r="AN2" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="AO2" s="29" t="s">
+      <c r="AO2" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="AP2" s="32" t="s">
+      <c r="AP2" s="45" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:42" s="5" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="42"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="53"/>
-      <c r="G3" s="53"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="35" t="s">
+      <c r="B3" s="28"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="42" t="s">
+      <c r="J3" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="36" t="s">
+      <c r="K3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="39" t="s">
+      <c r="L3" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="M3" s="42" t="s">
+      <c r="M3" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="42"/>
-      <c r="O3" s="42"/>
-      <c r="P3" s="42"/>
-      <c r="Q3" s="28" t="s">
+      <c r="N3" s="28"/>
+      <c r="O3" s="28"/>
+      <c r="P3" s="28"/>
+      <c r="Q3" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="R3" s="28" t="s">
+      <c r="R3" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="S3" s="28" t="s">
+      <c r="S3" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="T3" s="28" t="s">
+      <c r="T3" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="U3" s="28" t="s">
+      <c r="U3" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="V3" s="28" t="s">
+      <c r="V3" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="46"/>
-      <c r="X3" s="30"/>
-      <c r="Y3" s="33"/>
-      <c r="Z3" s="35" t="s">
+      <c r="W3" s="49"/>
+      <c r="X3" s="38"/>
+      <c r="Y3" s="46"/>
+      <c r="Z3" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="AA3" s="42" t="s">
+      <c r="AA3" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="AB3" s="36" t="s">
+      <c r="AB3" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="AC3" s="39" t="s">
+      <c r="AC3" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="AD3" s="42" t="s">
+      <c r="AD3" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="AE3" s="42"/>
-      <c r="AF3" s="42"/>
-      <c r="AG3" s="42"/>
-      <c r="AH3" s="28" t="s">
+      <c r="AE3" s="28"/>
+      <c r="AF3" s="28"/>
+      <c r="AG3" s="28"/>
+      <c r="AH3" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="AI3" s="28" t="s">
+      <c r="AI3" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="AJ3" s="28" t="s">
+      <c r="AJ3" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="AK3" s="28" t="s">
+      <c r="AK3" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="AL3" s="28" t="s">
+      <c r="AL3" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="AM3" s="28" t="s">
+      <c r="AM3" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="AN3" s="46"/>
-      <c r="AO3" s="30"/>
-      <c r="AP3" s="33"/>
+      <c r="AN3" s="49"/>
+      <c r="AO3" s="38"/>
+      <c r="AP3" s="46"/>
     </row>
     <row r="4" spans="1:42" s="5" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="B4" s="42"/>
-      <c r="C4" s="53"/>
-      <c r="D4" s="53"/>
-      <c r="E4" s="53"/>
-      <c r="F4" s="53"/>
-      <c r="G4" s="53"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="35"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="37"/>
-      <c r="L4" s="40"/>
-      <c r="M4" s="28" t="s">
+      <c r="B4" s="28"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="51"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="41"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="28" t="s">
+      <c r="P4" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="Q4" s="28"/>
-      <c r="R4" s="28"/>
-      <c r="S4" s="28"/>
-      <c r="T4" s="28"/>
-      <c r="U4" s="28"/>
-      <c r="V4" s="28"/>
-      <c r="W4" s="46"/>
-      <c r="X4" s="30"/>
-      <c r="Y4" s="33"/>
-      <c r="Z4" s="35"/>
-      <c r="AA4" s="42"/>
-      <c r="AB4" s="37"/>
-      <c r="AC4" s="40"/>
-      <c r="AD4" s="28" t="s">
+      <c r="Q4" s="35"/>
+      <c r="R4" s="35"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
+      <c r="W4" s="49"/>
+      <c r="X4" s="38"/>
+      <c r="Y4" s="46"/>
+      <c r="Z4" s="51"/>
+      <c r="AA4" s="28"/>
+      <c r="AB4" s="41"/>
+      <c r="AC4" s="53"/>
+      <c r="AD4" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="AE4" s="28" t="s">
+      <c r="AE4" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="AF4" s="28" t="s">
+      <c r="AF4" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="AG4" s="28" t="s">
+      <c r="AG4" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="AH4" s="28"/>
-      <c r="AI4" s="28"/>
-      <c r="AJ4" s="28"/>
-      <c r="AK4" s="28"/>
-      <c r="AL4" s="28"/>
-      <c r="AM4" s="28"/>
-      <c r="AN4" s="46"/>
-      <c r="AO4" s="30"/>
-      <c r="AP4" s="33"/>
+      <c r="AH4" s="35"/>
+      <c r="AI4" s="35"/>
+      <c r="AJ4" s="35"/>
+      <c r="AK4" s="35"/>
+      <c r="AL4" s="35"/>
+      <c r="AM4" s="35"/>
+      <c r="AN4" s="49"/>
+      <c r="AO4" s="38"/>
+      <c r="AP4" s="46"/>
     </row>
     <row r="5" spans="1:42" s="5" customFormat="1" ht="99.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="54"/>
-      <c r="D5" s="54"/>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="35"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="28"/>
-      <c r="R5" s="28"/>
-      <c r="S5" s="28"/>
-      <c r="T5" s="28"/>
-      <c r="U5" s="28"/>
-      <c r="V5" s="28"/>
-      <c r="W5" s="47"/>
-      <c r="X5" s="31"/>
-      <c r="Y5" s="34"/>
-      <c r="Z5" s="35"/>
-      <c r="AA5" s="42"/>
-      <c r="AB5" s="38"/>
-      <c r="AC5" s="41"/>
-      <c r="AD5" s="28"/>
-      <c r="AE5" s="28"/>
-      <c r="AF5" s="28"/>
-      <c r="AG5" s="28"/>
-      <c r="AH5" s="28"/>
-      <c r="AI5" s="28"/>
-      <c r="AJ5" s="28"/>
-      <c r="AK5" s="28"/>
-      <c r="AL5" s="28"/>
-      <c r="AM5" s="28"/>
-      <c r="AN5" s="47"/>
-      <c r="AO5" s="31"/>
-      <c r="AP5" s="34"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="31"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="51"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="35"/>
+      <c r="N5" s="35"/>
+      <c r="O5" s="35"/>
+      <c r="P5" s="35"/>
+      <c r="Q5" s="35"/>
+      <c r="R5" s="35"/>
+      <c r="S5" s="35"/>
+      <c r="T5" s="35"/>
+      <c r="U5" s="35"/>
+      <c r="V5" s="35"/>
+      <c r="W5" s="50"/>
+      <c r="X5" s="39"/>
+      <c r="Y5" s="47"/>
+      <c r="Z5" s="51"/>
+      <c r="AA5" s="28"/>
+      <c r="AB5" s="42"/>
+      <c r="AC5" s="54"/>
+      <c r="AD5" s="35"/>
+      <c r="AE5" s="35"/>
+      <c r="AF5" s="35"/>
+      <c r="AG5" s="35"/>
+      <c r="AH5" s="35"/>
+      <c r="AI5" s="35"/>
+      <c r="AJ5" s="35"/>
+      <c r="AK5" s="35"/>
+      <c r="AL5" s="35"/>
+      <c r="AM5" s="35"/>
+      <c r="AN5" s="50"/>
+      <c r="AO5" s="39"/>
+      <c r="AP5" s="47"/>
     </row>
     <row r="6" spans="1:42" s="5" customFormat="1" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
@@ -9235,7 +9235,9 @@
       <c r="AP19" s="27"/>
     </row>
     <row r="20" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="13"/>
+      <c r="B20" s="13">
+        <v>14</v>
+      </c>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
@@ -9299,7 +9301,7 @@
     </row>
     <row r="21" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="13">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
@@ -9364,7 +9366,7 @@
     </row>
     <row r="22" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="13">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
@@ -9429,7 +9431,7 @@
     </row>
     <row r="23" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="13">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
@@ -9494,7 +9496,7 @@
     </row>
     <row r="24" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="13">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
@@ -9559,7 +9561,7 @@
     </row>
     <row r="25" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="13">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C25" s="14"/>
       <c r="D25" s="14"/>
@@ -9624,7 +9626,7 @@
     </row>
     <row r="26" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="13">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
@@ -9689,7 +9691,7 @@
     </row>
     <row r="27" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="13">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
@@ -9754,7 +9756,7 @@
     </row>
     <row r="28" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="13">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
@@ -9818,7 +9820,9 @@
       <c r="AP28" s="27"/>
     </row>
     <row r="29" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="13"/>
+      <c r="B29" s="13">
+        <v>23</v>
+      </c>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
@@ -9882,7 +9886,7 @@
     </row>
     <row r="30" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="13">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
@@ -9947,7 +9951,7 @@
     </row>
     <row r="31" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="13">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
@@ -10012,7 +10016,7 @@
     </row>
     <row r="32" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="13">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
@@ -10077,7 +10081,7 @@
     </row>
     <row r="33" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="13">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
@@ -10142,7 +10146,7 @@
     </row>
     <row r="34" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="13">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C34" s="14"/>
       <c r="D34" s="14"/>
@@ -10207,7 +10211,7 @@
     </row>
     <row r="35" spans="2:42" s="12" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="13">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
@@ -10272,7 +10276,7 @@
     </row>
     <row r="36" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="13">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C36" s="14"/>
       <c r="D36" s="14"/>
@@ -10337,7 +10341,7 @@
     </row>
     <row r="37" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="13">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C37" s="14"/>
       <c r="D37" s="14"/>
@@ -10402,7 +10406,7 @@
     </row>
     <row r="38" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="13">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C38" s="14"/>
       <c r="D38" s="14"/>
@@ -10467,7 +10471,7 @@
     </row>
     <row r="39" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="13">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C39" s="14"/>
       <c r="D39" s="14"/>
@@ -10532,7 +10536,7 @@
     </row>
     <row r="40" spans="2:42" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="13">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
@@ -10597,7 +10601,7 @@
     </row>
     <row r="41" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="13">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C41" s="14"/>
       <c r="D41" s="14"/>
@@ -10662,7 +10666,7 @@
     </row>
     <row r="42" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="13">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C42" s="14"/>
       <c r="D42" s="14"/>
@@ -10727,7 +10731,7 @@
     </row>
     <row r="43" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="13">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C43" s="14"/>
       <c r="D43" s="14"/>
@@ -10792,7 +10796,7 @@
     </row>
     <row r="44" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="13">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
@@ -10857,7 +10861,7 @@
     </row>
     <row r="45" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="13">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C45" s="14"/>
       <c r="D45" s="14"/>
@@ -10922,7 +10926,7 @@
     </row>
     <row r="46" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="13">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C46" s="14"/>
       <c r="D46" s="14"/>
@@ -10987,7 +10991,7 @@
     </row>
     <row r="47" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="13">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C47" s="14"/>
       <c r="D47" s="14"/>
@@ -11052,7 +11056,7 @@
     </row>
     <row r="48" spans="2:42" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="13">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C48" s="14"/>
       <c r="D48" s="14"/>
@@ -11117,7 +11121,7 @@
     </row>
     <row r="49" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="13">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C49" s="14"/>
       <c r="D49" s="14"/>
@@ -11182,7 +11186,7 @@
     </row>
     <row r="50" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="13">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C50" s="14"/>
       <c r="D50" s="14"/>
@@ -11247,7 +11251,7 @@
     </row>
     <row r="51" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="13">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C51" s="14"/>
       <c r="D51" s="14"/>
@@ -11312,7 +11316,7 @@
     </row>
     <row r="52" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="13">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C52" s="14"/>
       <c r="D52" s="14"/>
@@ -11377,7 +11381,7 @@
     </row>
     <row r="53" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="13">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C53" s="14"/>
       <c r="D53" s="14"/>
@@ -11442,7 +11446,7 @@
     </row>
     <row r="54" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="13">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C54" s="14"/>
       <c r="D54" s="14"/>
@@ -11507,7 +11511,7 @@
     </row>
     <row r="55" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="13">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C55" s="14"/>
       <c r="D55" s="14"/>
@@ -11572,7 +11576,7 @@
     </row>
     <row r="56" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="13">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C56" s="14"/>
       <c r="D56" s="14"/>
@@ -11637,7 +11641,7 @@
     </row>
     <row r="57" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="13">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C57" s="14"/>
       <c r="D57" s="14"/>
@@ -11702,7 +11706,7 @@
     </row>
     <row r="58" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="13">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C58" s="14"/>
       <c r="D58" s="14"/>
@@ -11767,7 +11771,7 @@
     </row>
     <row r="59" spans="2:42" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="13">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C59" s="14"/>
       <c r="D59" s="14"/>
@@ -11832,7 +11836,7 @@
     </row>
     <row r="60" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="13">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C60" s="14"/>
       <c r="D60" s="14"/>
@@ -11897,7 +11901,7 @@
     </row>
     <row r="61" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="13">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C61" s="14"/>
       <c r="D61" s="14"/>
@@ -11962,7 +11966,7 @@
     </row>
     <row r="62" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="13">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C62" s="14"/>
       <c r="D62" s="14"/>
@@ -12027,7 +12031,7 @@
     </row>
     <row r="63" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="13">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
@@ -12092,7 +12096,7 @@
     </row>
     <row r="64" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="13">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C64" s="14"/>
       <c r="D64" s="14"/>
@@ -12157,7 +12161,7 @@
     </row>
     <row r="65" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="13">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C65" s="14"/>
       <c r="D65" s="14"/>
@@ -12222,7 +12226,7 @@
     </row>
     <row r="66" spans="2:42" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="13">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C66" s="14"/>
       <c r="D66" s="14"/>
@@ -12287,7 +12291,7 @@
     </row>
     <row r="67" spans="2:42" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="13">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C67" s="14"/>
       <c r="D67" s="14"/>
@@ -12353,41 +12357,6 @@
   </sheetData>
   <autoFilter ref="B6:Y67" xr:uid="{00000000-0009-0000-0000-00001B000000}"/>
   <mergeCells count="46">
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="Q3:Q5"/>
-    <mergeCell ref="T3:T5"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="G1:Y1"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="X2:X5"/>
-    <mergeCell ref="K3:K5"/>
-    <mergeCell ref="Z2:AM2"/>
-    <mergeCell ref="Y2:Y5"/>
-    <mergeCell ref="W2:W5"/>
-    <mergeCell ref="AG4:AG5"/>
-    <mergeCell ref="AD4:AD5"/>
-    <mergeCell ref="AE4:AE5"/>
-    <mergeCell ref="AF4:AF5"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="O4:O5"/>
-    <mergeCell ref="AA3:AA5"/>
-    <mergeCell ref="S3:S5"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="U3:U5"/>
-    <mergeCell ref="I2:V2"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="L3:L5"/>
-    <mergeCell ref="R3:R5"/>
-    <mergeCell ref="J3:J5"/>
-    <mergeCell ref="AL3:AL5"/>
-    <mergeCell ref="AM3:AM5"/>
     <mergeCell ref="AO2:AO5"/>
     <mergeCell ref="AP2:AP5"/>
     <mergeCell ref="Z3:Z5"/>
@@ -12399,6 +12368,41 @@
     <mergeCell ref="AJ3:AJ5"/>
     <mergeCell ref="AK3:AK5"/>
     <mergeCell ref="AN2:AN5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="L3:L5"/>
+    <mergeCell ref="R3:R5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="AL3:AL5"/>
+    <mergeCell ref="Z2:AM2"/>
+    <mergeCell ref="Y2:Y5"/>
+    <mergeCell ref="W2:W5"/>
+    <mergeCell ref="AG4:AG5"/>
+    <mergeCell ref="AD4:AD5"/>
+    <mergeCell ref="AE4:AE5"/>
+    <mergeCell ref="AF4:AF5"/>
+    <mergeCell ref="AA3:AA5"/>
+    <mergeCell ref="AM3:AM5"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="Q3:Q5"/>
+    <mergeCell ref="T3:T5"/>
+    <mergeCell ref="V3:V5"/>
+    <mergeCell ref="G1:Y1"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="X2:X5"/>
+    <mergeCell ref="K3:K5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="S3:S5"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="U3:U5"/>
+    <mergeCell ref="I2:V2"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="F2:F5"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>